<commit_message>
add import function and excel template
</commit_message>
<xml_diff>
--- a/data/Swisscom Bedag Stadt-ZRH.xlsx
+++ b/data/Swisscom Bedag Stadt-ZRH.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Red Hat Contract</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -471,17 +471,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>automation</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>On Track</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
+          <t>&lt;p&gt;check&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -491,7 +491,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Test 2</t>
+          <t>Postgres on VM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -501,17 +501,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>edge-platforms</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>On Track</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>&lt;p&gt;check&lt;/p&gt;</t>
+          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -521,32 +521,62 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Test Tags!</t>
+          <t>Data Opportunity</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ready</t>
+          <t>3+ Years</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>On Track</t>
+          <t>At Risk</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>&lt;p&gt;example&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TWS Replacement</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1-3 Years</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>automation</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>